<commit_message>
created module display.py with ASCII and COLOUR helpers
</commit_message>
<xml_diff>
--- a/crypto_options_trade_tracker.xlsx
+++ b/crypto_options_trade_tracker.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -93,6 +93,11 @@
     <font>
       <name val="Arial"/>
       <color rgb="0027AE60"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00E8E8E8"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -189,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -243,6 +248,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1168,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N4"/>
+  <dimension ref="B2:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1313,6 +1327,51 @@
       <c r="N4" s="16" t="inlineStr">
         <is>
           <t>Held to expiry</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>Short Strangle — Open</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>2090</v>
+      </c>
+      <c r="E5" s="22" t="n">
+        <v>2550</v>
+      </c>
+      <c r="F5" s="23" t="n">
+        <v>2319.36</v>
+      </c>
+      <c r="G5" s="23" t="inlineStr"/>
+      <c r="H5" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="23" t="n">
+        <v>0.06560000000000001</v>
+      </c>
+      <c r="J5" s="22" t="inlineStr"/>
+      <c r="K5" s="22" t="n">
+        <v>2089.391399936</v>
+      </c>
+      <c r="L5" s="21" t="n">
+        <v>2550.608600064</v>
+      </c>
+      <c r="M5" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N5" s="21" t="inlineStr">
+        <is>
+          <t>Paper strangle, 1d expiry</t>
         </is>
       </c>
     </row>

</xml_diff>